<commit_message>
Day 3 completed - Dashboard and Analysis
</commit_message>
<xml_diff>
--- a/Excel/Pinterest_Analytics_Project.xlsx.xlsx
+++ b/Excel/Pinterest_Analytics_Project.xlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/afea116efc88aa0e/Desktop/Pinterest-Analytics-Project/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="569" documentId="11_F25DC773A252ABDACC104889019A7CC25BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6A5220A-F0AB-4D4B-9051-2D9E5D027FB1}"/>
+  <xr:revisionPtr revIDLastSave="570" documentId="11_F25DC773A252ABDACC104889019A7CC25BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2044FF0E-E3BB-4A3F-A79C-36939E8284B3}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -88,9 +88,6 @@
     <t>Basic Excel</t>
   </si>
   <si>
-    <t>Day 1</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -323,6 +320,9 @@
   </si>
   <si>
     <t>Focus future  pinterest pins on lunch box products</t>
+  </si>
+  <si>
+    <t>Day 1&amp;2</t>
   </si>
 </sst>
 </file>
@@ -744,6 +744,9 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -751,9 +754,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2515,10 +2515,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2857,7 +2853,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>15</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -2876,40 +2872,40 @@
   <sheetData>
     <row r="1" spans="1:19" s="11" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="C1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D1" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="E1" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="F1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="G1" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="H1" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="J1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="K1" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="L1" s="11" t="s">
         <v>25</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="11" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2917,19 +2913,19 @@
         <v>46204</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G2" s="15">
         <v>499</v>
@@ -2962,19 +2958,19 @@
         <v>46204</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G3" s="15">
         <v>399</v>
@@ -3007,19 +3003,19 @@
         <v>46204</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G4" s="15">
         <v>399</v>
@@ -3052,19 +3048,19 @@
         <v>46205</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G5" s="15">
         <v>399</v>
@@ -3097,19 +3093,19 @@
         <v>46205</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G6" s="15">
         <v>399</v>
@@ -3142,19 +3138,19 @@
         <v>46205</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G7" s="15">
         <v>399</v>
@@ -3187,19 +3183,19 @@
         <v>46206</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G8" s="15">
         <v>399</v>
@@ -3232,19 +3228,19 @@
         <v>46206</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G9" s="15">
         <v>699</v>
@@ -3277,19 +3273,19 @@
         <v>46206</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G10" s="15">
         <v>699</v>
@@ -3322,19 +3318,19 @@
         <v>46206</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="G11" s="15">
         <v>699</v>
@@ -3423,57 +3419,57 @@
   <sheetData>
     <row r="1" spans="1:2" s="16" customFormat="1" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>59</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:2" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" s="1"/>
     </row>
     <row r="4" spans="1:2" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5" spans="1:2" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B5" s="1"/>
     </row>
     <row r="6" spans="1:2" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B6" s="1"/>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B7" s="1"/>
     </row>
     <row r="8" spans="1:2" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B8" s="1"/>
     </row>
     <row r="9" spans="1:2" ht="26.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B9" s="1"/>
     </row>
@@ -3497,18 +3493,18 @@
   <sheetData>
     <row r="1" spans="1:4" s="17" customFormat="1" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="18" t="s">
         <v>61</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B2" s="20">
         <f>COUNTIF(Raw_Data!C:C,A2)</f>
@@ -3521,7 +3517,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3" s="23">
         <f>COUNTIF(Raw_Data!C:C,A3)</f>
@@ -3534,7 +3530,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B4" s="23">
         <f>COUNTIF(Raw_Data!C:C,A4)</f>
@@ -3547,7 +3543,7 @@
     </row>
     <row r="5" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" s="26">
         <f>COUNTIF(Raw_Data!C:C,A5)</f>
@@ -3560,7 +3556,7 @@
     </row>
     <row r="7" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B7" s="28"/>
       <c r="C7" s="28"/>
@@ -3568,7 +3564,7 @@
     </row>
     <row r="8" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B8" s="28"/>
       <c r="C8" s="28"/>
@@ -3576,7 +3572,7 @@
     </row>
     <row r="9" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B9" s="28"/>
       <c r="C9" s="28"/>
@@ -3600,18 +3596,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="29" t="s">
         <v>61</v>
-      </c>
-      <c r="C1" s="29" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2">
         <f>COUNTIF(Raw_Data!F:F,A2)</f>
@@ -3624,7 +3620,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B3">
         <f>COUNTIF(Raw_Data!F:F,A3)</f>
@@ -3637,7 +3633,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B4">
         <f>COUNTIF(Raw_Data!F:F,A4)</f>
@@ -3650,62 +3646,62 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -3723,26 +3719,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" s="37" customFormat="1" ht="35.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="38" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
+      <c r="A1" s="39" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="2" spans="1:20" ht="21" x14ac:dyDescent="0.5">
       <c r="A2" s="31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B2" s="32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B3" s="34">
         <f>COUNTA(Raw_Data!B2:B13)</f>
@@ -3751,7 +3747,7 @@
     </row>
     <row r="4" spans="1:20" ht="21" x14ac:dyDescent="0.35">
       <c r="A4" s="33" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B4" s="34">
         <f>SUM(Raw_Data!I2:I11)</f>
@@ -3760,96 +3756,96 @@
     </row>
     <row r="5" spans="1:20" ht="21" x14ac:dyDescent="0.35">
       <c r="A5" s="33" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="26" x14ac:dyDescent="0.6">
       <c r="A6" s="33" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B6" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="J6" s="39" t="s">
-        <v>89</v>
-      </c>
-      <c r="K6" s="40"/>
-      <c r="L6" s="40"/>
-      <c r="M6" s="40"/>
-      <c r="N6" s="40"/>
-      <c r="O6" s="40"/>
-      <c r="P6" s="40"/>
-      <c r="Q6" s="40"/>
-      <c r="R6" s="40"/>
-      <c r="S6" s="40"/>
-      <c r="T6" s="40"/>
+        <v>56</v>
+      </c>
+      <c r="J6" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="41"/>
+      <c r="O6" s="41"/>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="41"/>
+      <c r="R6" s="41"/>
+      <c r="S6" s="41"/>
+      <c r="T6" s="41"/>
     </row>
     <row r="7" spans="1:20" ht="24" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A7" s="35"/>
       <c r="B7" s="36"/>
-      <c r="J7" s="41" t="s">
-        <v>91</v>
-      </c>
-      <c r="K7" s="41"/>
-      <c r="L7" s="41"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="41"/>
-      <c r="P7" s="41"/>
-      <c r="Q7" s="41"/>
-      <c r="R7" s="41"/>
-      <c r="S7" s="41"/>
-      <c r="T7" s="41"/>
+      <c r="J7" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="K7" s="38"/>
+      <c r="L7" s="38"/>
+      <c r="M7" s="38"/>
+      <c r="N7" s="38"/>
+      <c r="O7" s="38"/>
+      <c r="P7" s="38"/>
+      <c r="Q7" s="38"/>
+      <c r="R7" s="38"/>
+      <c r="S7" s="38"/>
+      <c r="T7" s="38"/>
     </row>
     <row r="8" spans="1:20" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30"/>
       <c r="B8" s="30"/>
-      <c r="J8" s="41" t="s">
-        <v>90</v>
-      </c>
-      <c r="K8" s="41"/>
-      <c r="L8" s="41"/>
-      <c r="M8" s="41"/>
-      <c r="N8" s="41"/>
-      <c r="O8" s="41"/>
-      <c r="P8" s="41"/>
-      <c r="Q8" s="41"/>
-      <c r="R8" s="41"/>
-      <c r="S8" s="41"/>
-      <c r="T8" s="41"/>
+      <c r="J8" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="K8" s="38"/>
+      <c r="L8" s="38"/>
+      <c r="M8" s="38"/>
+      <c r="N8" s="38"/>
+      <c r="O8" s="38"/>
+      <c r="P8" s="38"/>
+      <c r="Q8" s="38"/>
+      <c r="R8" s="38"/>
+      <c r="S8" s="38"/>
+      <c r="T8" s="38"/>
     </row>
     <row r="9" spans="1:20" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="J9" s="41" t="s">
+      <c r="J9" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="K9" s="38"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="38"/>
+      <c r="N9" s="38"/>
+      <c r="O9" s="38"/>
+      <c r="P9" s="38"/>
+      <c r="Q9" s="38"/>
+      <c r="R9" s="38"/>
+      <c r="S9" s="38"/>
+      <c r="T9" s="38"/>
+    </row>
+    <row r="10" spans="1:20" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="J10" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="K9" s="41"/>
-      <c r="L9" s="41"/>
-      <c r="M9" s="41"/>
-      <c r="N9" s="41"/>
-      <c r="O9" s="41"/>
-      <c r="P9" s="41"/>
-      <c r="Q9" s="41"/>
-      <c r="R9" s="41"/>
-      <c r="S9" s="41"/>
-      <c r="T9" s="41"/>
-    </row>
-    <row r="10" spans="1:20" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="J10" s="41" t="s">
-        <v>93</v>
-      </c>
-      <c r="K10" s="41"/>
-      <c r="L10" s="41"/>
-      <c r="M10" s="41"/>
-      <c r="N10" s="41"/>
-      <c r="O10" s="41"/>
-      <c r="P10" s="41"/>
-      <c r="Q10" s="41"/>
-      <c r="R10" s="41"/>
-      <c r="S10" s="41"/>
-      <c r="T10" s="41"/>
+      <c r="K10" s="38"/>
+      <c r="L10" s="38"/>
+      <c r="M10" s="38"/>
+      <c r="N10" s="38"/>
+      <c r="O10" s="38"/>
+      <c r="P10" s="38"/>
+      <c r="Q10" s="38"/>
+      <c r="R10" s="38"/>
+      <c r="S10" s="38"/>
+      <c r="T10" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>